<commit_message>
validation & Chronolofy chnages are done . !
</commit_message>
<xml_diff>
--- a/scratch/debug_out.xlsx
+++ b/scratch/debug_out.xlsx
@@ -144,7 +144,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -231,6 +231,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -740,27 +746,27 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AD39"/>
+  <dimension ref="A1:AD32"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.5703125" defaultRowHeight="42.95" customHeight="1"/>
   <cols>
-    <col width="7.7109375" customWidth="1" style="29" min="1" max="1"/>
-    <col width="25.42578125" customWidth="1" style="29" min="2" max="2"/>
-    <col width="28.28515625" customWidth="1" style="29" min="3" max="3"/>
-    <col width="22.42578125" customWidth="1" style="29" min="4" max="4"/>
-    <col width="18.5703125" customWidth="1" style="29" min="5" max="5"/>
-    <col width="30.85546875" customWidth="1" style="29" min="6" max="6"/>
-    <col width="28.5703125" customWidth="1" style="29" min="7" max="7"/>
-    <col width="22.7109375" customWidth="1" style="29" min="8" max="8"/>
-    <col width="30.28515625" customWidth="1" style="29" min="9" max="9"/>
-    <col width="25.85546875" customWidth="1" style="29" min="10" max="10"/>
-    <col width="20.85546875" customWidth="1" style="29" min="11" max="11"/>
-    <col width="21.7109375" customWidth="1" style="29" min="12" max="12"/>
-    <col width="17" customWidth="1" style="29" min="13" max="13"/>
-    <col width="20.5703125" customWidth="1" style="29" min="14" max="14"/>
-    <col width="21.5703125" customWidth="1" style="29" min="15" max="15"/>
-    <col width="19.28515625" customWidth="1" style="29" min="16" max="16"/>
+    <col width="7.7" customWidth="1" style="29" min="1" max="1"/>
+    <col width="24.92" customWidth="1" style="29" min="2" max="2"/>
+    <col width="27.72" customWidth="1" style="29" min="3" max="3"/>
+    <col width="6" customWidth="1" style="29" min="4" max="4"/>
+    <col width="8.65" customWidth="1" style="29" min="5" max="5"/>
+    <col width="30.24" customWidth="1" style="29" min="6" max="6"/>
+    <col width="8.65" customWidth="1" style="29" min="7" max="7"/>
+    <col width="7.7" customWidth="1" style="29" min="8" max="8"/>
+    <col width="29.68" customWidth="1" style="29" min="9" max="9"/>
+    <col width="11.5" customWidth="1" style="29" min="10" max="10"/>
+    <col width="11.5" customWidth="1" style="29" min="11" max="11"/>
+    <col width="9.6" customWidth="1" style="29" min="12" max="12"/>
+    <col width="11.5" customWidth="1" style="29" min="13" max="13"/>
+    <col width="13.4" customWidth="1" style="29" min="14" max="14"/>
+    <col width="13.4" customWidth="1" style="29" min="15" max="15"/>
+    <col width="7.7" customWidth="1" style="29" min="16" max="16"/>
     <col width="11.5703125" customWidth="1" style="29" min="17" max="252"/>
   </cols>
   <sheetData>
@@ -799,7 +805,7 @@
     <row r="5" ht="13.35" customFormat="1" customHeight="1" s="4">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>Product Series :</t>
+          <t>Product Series:</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -807,315 +813,303 @@
           <t>LPRS480</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n"/>
-      <c r="D5" s="7" t="n"/>
-      <c r="E5" s="7" t="n"/>
-      <c r="F5" s="7" t="n"/>
-      <c r="G5" s="7" t="n"/>
-      <c r="H5" s="7" t="n"/>
-      <c r="I5" s="7" t="n"/>
-      <c r="J5" s="7" t="n"/>
-      <c r="K5" s="9" t="n"/>
-      <c r="L5" s="9" t="n"/>
-      <c r="M5" s="9" t="n"/>
-      <c r="N5" s="9" t="n"/>
-      <c r="O5" s="9" t="n"/>
-      <c r="P5" s="9" t="n"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr"/>
+      <c r="I5" s="7" t="inlineStr"/>
+      <c r="J5" s="7" t="inlineStr"/>
+      <c r="K5" s="9" t="inlineStr"/>
+      <c r="L5" s="9" t="inlineStr"/>
+      <c r="M5" s="9" t="inlineStr"/>
+      <c r="N5" s="9" t="inlineStr"/>
+      <c r="O5" s="9" t="inlineStr"/>
+      <c r="P5" s="9" t="inlineStr"/>
     </row>
     <row r="6" ht="13.35" customFormat="1" customHeight="1" s="4">
-      <c r="A6" s="30" t="inlineStr">
-        <is>
-          <t>Applicable Products:</t>
-        </is>
-      </c>
-      <c r="K6" s="9" t="n"/>
-      <c r="L6" s="9" t="n"/>
-      <c r="M6" s="9" t="n"/>
-      <c r="N6" s="9" t="n"/>
-      <c r="O6" s="9" t="n"/>
-      <c r="P6" s="9" t="n"/>
+      <c r="A6" s="30" t="inlineStr"/>
+      <c r="K6" s="9" t="inlineStr"/>
+      <c r="L6" s="9" t="inlineStr"/>
+      <c r="M6" s="9" t="inlineStr"/>
+      <c r="N6" s="9" t="inlineStr"/>
+      <c r="O6" s="9" t="inlineStr"/>
+      <c r="P6" s="9" t="inlineStr"/>
     </row>
     <row r="7" ht="12.75" customFormat="1" customHeight="1" s="4">
-      <c r="A7" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>LRPS480-24-CE</t>
-        </is>
-      </c>
-      <c r="C7" s="9" t="n"/>
-      <c r="D7" s="9" t="n"/>
-      <c r="E7" s="9" t="n"/>
-      <c r="F7" s="9" t="n"/>
-      <c r="G7" s="9" t="n"/>
-      <c r="H7" s="9" t="n"/>
-      <c r="I7" s="9" t="n"/>
-      <c r="J7" s="9" t="n"/>
-      <c r="K7" s="11" t="n"/>
-      <c r="L7" s="11" t="n"/>
-      <c r="M7" s="11" t="n"/>
-      <c r="N7" s="11" t="n"/>
-      <c r="O7" s="11" t="n"/>
-      <c r="P7" s="11" t="n"/>
+      <c r="A7" s="9" t="inlineStr"/>
+      <c r="B7" s="9" t="inlineStr"/>
+      <c r="C7" s="9" t="inlineStr"/>
+      <c r="D7" s="9" t="inlineStr"/>
+      <c r="E7" s="9" t="inlineStr"/>
+      <c r="F7" s="9" t="inlineStr"/>
+      <c r="G7" s="9" t="inlineStr"/>
+      <c r="H7" s="9" t="inlineStr"/>
+      <c r="I7" s="9" t="inlineStr"/>
+      <c r="J7" s="9" t="inlineStr"/>
+      <c r="K7" s="11" t="inlineStr"/>
+      <c r="L7" s="11" t="inlineStr"/>
+      <c r="M7" s="11" t="inlineStr"/>
+      <c r="N7" s="11" t="inlineStr"/>
+      <c r="O7" s="11" t="inlineStr"/>
+      <c r="P7" s="11" t="inlineStr"/>
     </row>
     <row r="8" ht="14.25" customFormat="1" customHeight="1" s="4">
       <c r="A8" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>LRPS480-24-CE</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr"/>
+      <c r="D8" s="9" t="inlineStr"/>
+      <c r="E8" s="9" t="inlineStr"/>
+      <c r="F8" s="9" t="inlineStr"/>
+      <c r="G8" s="9" t="inlineStr"/>
+      <c r="H8" s="9" t="inlineStr"/>
+      <c r="I8" s="9" t="inlineStr"/>
+      <c r="J8" s="9" t="inlineStr"/>
+      <c r="K8" s="11" t="inlineStr"/>
+      <c r="L8" s="11" t="inlineStr"/>
+      <c r="M8" s="11" t="inlineStr"/>
+      <c r="N8" s="11" t="inlineStr"/>
+      <c r="O8" s="11" t="inlineStr"/>
+      <c r="P8" s="11" t="inlineStr"/>
+    </row>
+    <row r="9" ht="12.75" customFormat="1" customHeight="1" s="4">
+      <c r="A9" s="9" t="inlineStr"/>
+      <c r="B9" s="9" t="inlineStr"/>
+      <c r="C9" s="9" t="inlineStr"/>
+      <c r="D9" s="9" t="inlineStr"/>
+      <c r="E9" s="9" t="inlineStr"/>
+      <c r="F9" s="9" t="inlineStr"/>
+      <c r="G9" s="9" t="inlineStr"/>
+      <c r="H9" s="9" t="inlineStr"/>
+      <c r="I9" s="9" t="inlineStr"/>
+      <c r="J9" s="9" t="inlineStr"/>
+      <c r="K9" s="11" t="inlineStr"/>
+      <c r="L9" s="11" t="inlineStr"/>
+      <c r="M9" s="11" t="inlineStr"/>
+      <c r="N9" s="11" t="inlineStr"/>
+      <c r="O9" s="11" t="inlineStr"/>
+      <c r="P9" s="11" t="inlineStr"/>
+    </row>
+    <row r="10" ht="12.75" customFormat="1" customHeight="1" s="4">
+      <c r="A10" s="13" t="inlineStr"/>
+      <c r="B10" s="13" t="inlineStr"/>
+      <c r="C10" s="13" t="inlineStr"/>
+      <c r="D10" s="13" t="inlineStr"/>
+      <c r="E10" s="13" t="inlineStr"/>
+      <c r="F10" s="13" t="inlineStr"/>
+      <c r="G10" s="13" t="inlineStr"/>
+      <c r="H10" s="13" t="inlineStr"/>
+      <c r="I10" s="13" t="inlineStr"/>
+      <c r="J10" s="13" t="inlineStr"/>
+      <c r="K10" s="11" t="inlineStr"/>
+      <c r="L10" s="11" t="inlineStr"/>
+      <c r="M10" s="11" t="inlineStr"/>
+      <c r="N10" s="11" t="inlineStr"/>
+      <c r="O10" s="11" t="inlineStr"/>
+      <c r="P10" s="11" t="inlineStr"/>
+    </row>
+    <row r="11" ht="12.75" customHeight="1" s="2">
+      <c r="A11" s="9" t="inlineStr"/>
+      <c r="B11" s="9" t="inlineStr"/>
+      <c r="C11" s="9" t="inlineStr"/>
+      <c r="D11" s="9" t="inlineStr"/>
+      <c r="E11" s="9" t="inlineStr"/>
+      <c r="F11" s="9" t="inlineStr"/>
+      <c r="G11" s="9" t="inlineStr"/>
+      <c r="H11" s="9" t="inlineStr"/>
+      <c r="I11" s="9" t="inlineStr"/>
+      <c r="J11" s="9" t="inlineStr"/>
+      <c r="K11" s="15" t="inlineStr"/>
+      <c r="L11" s="15" t="inlineStr"/>
+      <c r="M11" s="15" t="inlineStr"/>
+      <c r="N11" s="15" t="inlineStr"/>
+      <c r="O11" s="15" t="inlineStr"/>
+      <c r="P11" s="15" t="inlineStr"/>
+    </row>
+    <row r="12" ht="12.75" customHeight="1" s="2">
+      <c r="A12" s="9" t="inlineStr"/>
+      <c r="B12" s="9" t="inlineStr"/>
+      <c r="C12" s="9" t="inlineStr"/>
+      <c r="D12" s="9" t="inlineStr"/>
+      <c r="E12" s="9" t="inlineStr"/>
+      <c r="F12" s="9" t="inlineStr"/>
+      <c r="G12" s="9" t="inlineStr"/>
+      <c r="H12" s="9" t="inlineStr"/>
+      <c r="I12" s="9" t="inlineStr"/>
+      <c r="J12" s="9" t="inlineStr"/>
+      <c r="K12" s="15" t="inlineStr"/>
+      <c r="L12" s="15" t="inlineStr"/>
+      <c r="M12" s="15" t="inlineStr"/>
+      <c r="N12" s="15" t="inlineStr"/>
+      <c r="O12" s="15" t="inlineStr"/>
+      <c r="P12" s="15" t="inlineStr"/>
+    </row>
+    <row r="13" ht="14.25" customHeight="1" s="2">
+      <c r="A13" s="16" t="inlineStr"/>
+      <c r="B13" s="16" t="inlineStr"/>
+      <c r="C13" s="16" t="inlineStr"/>
+      <c r="D13" s="16" t="inlineStr"/>
+      <c r="E13" s="16" t="inlineStr"/>
+      <c r="F13" s="16" t="inlineStr"/>
+      <c r="G13" s="16" t="inlineStr"/>
+      <c r="H13" s="16" t="inlineStr"/>
+      <c r="I13" s="16" t="inlineStr"/>
+      <c r="J13" s="16" t="inlineStr"/>
+      <c r="K13" s="16" t="inlineStr"/>
+      <c r="L13" s="16" t="inlineStr"/>
+      <c r="M13" s="16" t="inlineStr"/>
+      <c r="N13" s="16" t="inlineStr"/>
+      <c r="O13" s="16" t="inlineStr"/>
+      <c r="P13" s="16" t="inlineStr"/>
+    </row>
+    <row r="14" ht="54" customFormat="1" customHeight="1" s="29">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Serial No. </t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Source Code Path</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>Bin File Name</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="E14" s="18" t="inlineStr">
+        <is>
+          <t>Ladder Version No.</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>Reason For Upgrade</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>Testing Stage</t>
+        </is>
+      </c>
+      <c r="H14" s="19" t="inlineStr">
+        <is>
+          <t>PLC Model</t>
+        </is>
+      </c>
+      <c r="I14" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Selpro Version &amp; Path </t>
+        </is>
+      </c>
+      <c r="J14" s="18" t="inlineStr">
+        <is>
+          <t>Bootloader Version</t>
+        </is>
+      </c>
+      <c r="K14" s="18" t="inlineStr">
+        <is>
+          <t>Release Date</t>
+        </is>
+      </c>
+      <c r="L14" s="18" t="inlineStr">
+        <is>
+          <t>Released By</t>
+        </is>
+      </c>
+      <c r="M14" s="18" t="inlineStr">
+        <is>
+          <t>Ladder  Release – To Production</t>
+        </is>
+      </c>
+      <c r="N14" s="18" t="inlineStr">
+        <is>
+          <t>Operator Procedure Modification</t>
+        </is>
+      </c>
+      <c r="O14" s="18" t="inlineStr">
+        <is>
+          <t>Automation Set Up Modification</t>
+        </is>
+      </c>
+      <c r="P14" s="18" t="inlineStr">
+        <is>
+          <t>Tested By</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customFormat="1" customHeight="1" s="29">
+      <c r="A15" s="34" t="n">
         <v>2</v>
       </c>
-      <c r="B8" s="9" t="n"/>
-      <c r="C8" s="9" t="n"/>
-      <c r="D8" s="9" t="n"/>
-      <c r="E8" s="9" t="n"/>
-      <c r="F8" s="9" t="n"/>
-      <c r="G8" s="9" t="n"/>
-      <c r="H8" s="9" t="n"/>
-      <c r="I8" s="9" t="n"/>
-      <c r="J8" s="9" t="n"/>
-      <c r="K8" s="11" t="n"/>
-      <c r="L8" s="11" t="n"/>
-      <c r="M8" s="11" t="n"/>
-      <c r="N8" s="11" t="n"/>
-      <c r="O8" s="11" t="n"/>
-      <c r="P8" s="11" t="n"/>
-    </row>
-    <row r="9" ht="12.75" customFormat="1" customHeight="1" s="4">
-      <c r="A9" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="B9" s="9" t="n"/>
-      <c r="C9" s="9" t="n"/>
-      <c r="D9" s="9" t="n"/>
-      <c r="E9" s="9" t="n"/>
-      <c r="F9" s="9" t="n"/>
-      <c r="G9" s="9" t="n"/>
-      <c r="H9" s="9" t="n"/>
-      <c r="I9" s="9" t="n"/>
-      <c r="J9" s="9" t="n"/>
-      <c r="K9" s="11" t="n"/>
-      <c r="L9" s="11" t="n"/>
-      <c r="M9" s="11" t="n"/>
-      <c r="N9" s="11" t="n"/>
-      <c r="O9" s="11" t="n"/>
-      <c r="P9" s="11" t="n"/>
-    </row>
-    <row r="10" ht="12.75" customFormat="1" customHeight="1" s="4">
-      <c r="A10" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="B10" s="13" t="n"/>
-      <c r="C10" s="13" t="n"/>
-      <c r="D10" s="13" t="n"/>
-      <c r="E10" s="13" t="n"/>
-      <c r="F10" s="13" t="n"/>
-      <c r="G10" s="13" t="n"/>
-      <c r="H10" s="13" t="n"/>
-      <c r="I10" s="13" t="n"/>
-      <c r="J10" s="13" t="n"/>
-      <c r="K10" s="11" t="n"/>
-      <c r="L10" s="11" t="n"/>
-      <c r="M10" s="11" t="n"/>
-      <c r="N10" s="11" t="n"/>
-      <c r="O10" s="11" t="n"/>
-      <c r="P10" s="11" t="n"/>
-    </row>
-    <row r="11" ht="12.75" customHeight="1" s="2">
-      <c r="A11" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="B11" s="9" t="n"/>
-      <c r="C11" s="9" t="n"/>
-      <c r="D11" s="9" t="n"/>
-      <c r="E11" s="9" t="n"/>
-      <c r="F11" s="9" t="n"/>
-      <c r="G11" s="9" t="n"/>
-      <c r="H11" s="9" t="n"/>
-      <c r="I11" s="9" t="n"/>
-      <c r="J11" s="9" t="n"/>
-      <c r="K11" s="15" t="n"/>
-      <c r="L11" s="15" t="n"/>
-      <c r="M11" s="15" t="n"/>
-      <c r="N11" s="15" t="n"/>
-      <c r="O11" s="15" t="n"/>
-      <c r="P11" s="15" t="n"/>
-    </row>
-    <row r="12" ht="12.75" customHeight="1" s="2">
-      <c r="A12" s="9" t="n"/>
-      <c r="B12" s="9" t="n"/>
-      <c r="C12" s="9" t="n"/>
-      <c r="D12" s="9" t="n"/>
-      <c r="E12" s="9" t="n"/>
-      <c r="F12" s="9" t="n"/>
-      <c r="G12" s="9" t="n"/>
-      <c r="H12" s="9" t="n"/>
-      <c r="I12" s="9" t="n"/>
-      <c r="J12" s="9" t="n"/>
-      <c r="K12" s="15" t="n"/>
-      <c r="L12" s="15" t="n"/>
-      <c r="M12" s="15" t="n"/>
-      <c r="N12" s="15" t="n"/>
-      <c r="O12" s="15" t="n"/>
-      <c r="P12" s="15" t="n"/>
-    </row>
-    <row r="13" ht="14.25" customHeight="1" s="2">
-      <c r="A13" s="16" t="n"/>
-      <c r="B13" s="16" t="n"/>
-      <c r="C13" s="16" t="n"/>
-      <c r="D13" s="16" t="n"/>
-      <c r="E13" s="16" t="n"/>
-      <c r="F13" s="16" t="n"/>
-      <c r="G13" s="16" t="n"/>
-      <c r="H13" s="16" t="n"/>
-      <c r="I13" s="16" t="n"/>
-      <c r="J13" s="16" t="n"/>
-      <c r="K13" s="16" t="n"/>
-      <c r="L13" s="16" t="n"/>
-      <c r="M13" s="16" t="n"/>
-      <c r="N13" s="16" t="n"/>
-      <c r="O13" s="16" t="n"/>
-      <c r="P13" s="16" t="n"/>
-    </row>
-    <row r="14" ht="55.5" customFormat="1" customHeight="1" s="29">
-      <c r="A14" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Serial No. </t>
-        </is>
-      </c>
-      <c r="B14" s="18" t="inlineStr">
-        <is>
-          <t>Source Code Path</t>
-        </is>
-      </c>
-      <c r="C14" s="18" t="inlineStr">
-        <is>
-          <t>Bin File Name</t>
-        </is>
-      </c>
-      <c r="D14" s="18" t="inlineStr">
-        <is>
-          <t>CRC</t>
-        </is>
-      </c>
-      <c r="E14" s="18" t="inlineStr">
-        <is>
-          <t>Ladder Version No.</t>
-        </is>
-      </c>
-      <c r="F14" s="18" t="inlineStr">
-        <is>
-          <t>Reason For Upgrade</t>
-        </is>
-      </c>
-      <c r="G14" s="18" t="inlineStr">
-        <is>
-          <t>Testing Stage</t>
-        </is>
-      </c>
-      <c r="H14" s="19" t="inlineStr">
-        <is>
-          <t>PLC Model</t>
-        </is>
-      </c>
-      <c r="I14" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Selpro Version &amp; Path </t>
-        </is>
-      </c>
-      <c r="J14" s="18" t="inlineStr">
-        <is>
-          <t>Bootloader Version</t>
-        </is>
-      </c>
-      <c r="K14" s="18" t="inlineStr">
-        <is>
-          <t>Release Date</t>
-        </is>
-      </c>
-      <c r="L14" s="18" t="inlineStr">
-        <is>
-          <t>Released By</t>
-        </is>
-      </c>
-      <c r="M14" s="18" t="inlineStr">
-        <is>
-          <t>Ladder  Release – To Production</t>
-        </is>
-      </c>
-      <c r="N14" s="18" t="inlineStr">
-        <is>
-          <t>Operator Procedure Modification</t>
-        </is>
-      </c>
-      <c r="O14" s="18" t="inlineStr">
-        <is>
-          <t>Automation Set Up Modification</t>
-        </is>
-      </c>
-      <c r="P14" s="18" t="inlineStr">
-        <is>
-          <t>Tested By</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="112.35" customFormat="1" customHeight="1" s="29">
-      <c r="A15" s="21" t="n">
-        <v>2</v>
-      </c>
-      <c r="B15" s="22" t="inlineStr">
+      <c r="B15" s="35" t="inlineStr">
         <is>
           <t>dummy</t>
         </is>
       </c>
-      <c r="C15" s="22" t="inlineStr">
+      <c r="C15" s="35" t="inlineStr">
         <is>
           <t>dummy.bin</t>
         </is>
       </c>
-      <c r="D15" s="22" t="inlineStr">
+      <c r="D15" s="35" t="inlineStr">
         <is>
           <t>1234</t>
         </is>
       </c>
-      <c r="E15" s="22" t="inlineStr">
+      <c r="E15" s="35" t="inlineStr">
         <is>
           <t>V1.0</t>
         </is>
       </c>
-      <c r="F15" s="22" t="inlineStr">
+      <c r="F15" s="35" t="inlineStr">
         <is>
           <t>New feature</t>
         </is>
       </c>
-      <c r="G15" s="22" t="inlineStr">
+      <c r="G15" s="35" t="inlineStr">
         <is>
           <t>Initial</t>
         </is>
       </c>
-      <c r="H15" s="22" t="inlineStr">
+      <c r="H15" s="35" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="I15" s="22" t="inlineStr">
+      <c r="I15" s="35" t="inlineStr">
         <is>
           <t>V1</t>
         </is>
       </c>
-      <c r="J15" s="22" t="inlineStr">
+      <c r="J15" s="35" t="inlineStr">
         <is>
           <t>V1</t>
         </is>
       </c>
-      <c r="K15" s="22" t="inlineStr">
-        <is>
-          <t>06/08/2026</t>
-        </is>
-      </c>
-      <c r="L15" s="22" t="inlineStr"/>
-      <c r="M15" s="22" t="inlineStr"/>
-      <c r="N15" s="22" t="inlineStr"/>
-      <c r="O15" s="22" t="inlineStr"/>
-      <c r="P15" s="22" t="inlineStr"/>
+      <c r="K15" s="35" t="inlineStr">
+        <is>
+          <t>07/08/2026</t>
+        </is>
+      </c>
+      <c r="L15" s="35" t="inlineStr"/>
+      <c r="M15" s="35" t="inlineStr"/>
+      <c r="N15" s="35" t="inlineStr"/>
+      <c r="O15" s="35" t="inlineStr"/>
+      <c r="P15" s="35" t="inlineStr"/>
       <c r="Q15" s="23" t="n"/>
       <c r="R15" s="23" t="n"/>
       <c r="S15" s="23" t="n"/>
@@ -1131,11 +1125,11 @@
       <c r="AC15" s="23" t="n"/>
       <c r="AD15" s="23" t="n"/>
     </row>
-    <row r="16" ht="112.35" customHeight="1" s="2">
-      <c r="A16" s="21" t="n">
+    <row r="16" ht="20" customHeight="1" s="2">
+      <c r="A16" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="B16" s="31" t="inlineStr">
+      <c r="B16" s="35" t="inlineStr">
         <is>
           <t>bb</t>
         </is>
@@ -1438,26 +1432,19 @@
       <c r="O32" s="29" t="n"/>
       <c r="P32" s="29" t="n"/>
     </row>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A6:J6"/>
     <mergeCell ref="B16:P16"/>
   </mergeCells>
   <pageMargins left="0.7875" right="0.7875" top="1.549305555555555" bottom="0.8861111111111111" header="0.8861111111111111" footer="0.5118055555555555"/>
-  <pageSetup orientation="landscape" scale="33" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>
   <headerFooter alignWithMargins="0">
-    <oddHeader>&amp;L&amp;"Times New Roman,Regular"&amp;12 Selec Controls Pvt Ltd_x000a_DDHW_Department&amp;C&amp;"Times New Roman,Regular"&amp;12 Title- Ladder Release Chronology&amp;R&amp;"Times New Roman,Regular"&amp;12 FF/PM/DD-1120724     _x000a_Date :                               </oddHeader>
+    <oddHeader>&amp;L&amp;"Times New Roman,Regular"&amp;12 Selec Controls Pvt Ltd_x000a_DDHW_Department&amp;C&amp;"Times New Roman,Regular"&amp;12 Title- Ladder Release Chronology&amp;R&amp;"Times New Roman,Regular"&amp;12 FF/PM/DD-1120724_x000a_Date :</oddHeader>
     <oddFooter/>
-    <evenHeader/>
+    <evenHeader>&amp;L&amp;C&amp;R</evenHeader>
     <evenFooter/>
-    <firstHeader/>
+    <firstHeader>&amp;L&amp;C&amp;R</firstHeader>
     <firstFooter/>
   </headerFooter>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>